<commit_message>
Made few Changes related to Volumes
</commit_message>
<xml_diff>
--- a/datf_core/test/s2t/adls_adls_parquet_stage_removed.xlsx
+++ b/datf_core/test/s2t/adls_adls_parquet_stage_removed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajat.yadav\Downloads\McKesson\New Task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{008835C9-9266-4F67-93EA-D674AC8463DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D750C117-2FDA-424F-9CFE-A57137871235}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{60D25328-0517-4E51-B966-9D3337769260}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="122">
   <si>
     <t>mappingname</t>
   </si>
@@ -401,6 +401,9 @@
   </si>
   <si>
     <t>stagetimestampformat</t>
+  </si>
+  <si>
+    <t>raw_adls_connection</t>
   </si>
 </sst>
 </file>
@@ -482,16 +485,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -837,7 +836,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
-    <col min="2" max="2" width="88.7109375" style="4" customWidth="1"/>
+    <col min="2" max="2" width="88.7109375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -885,7 +884,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>101</v>
+        <v>121</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1034,8 +1033,8 @@
       <c r="A30" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B30" s="3" t="s">
-        <v>101</v>
+      <c r="B30" s="2" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1199,915 +1198,915 @@
   <dimension ref="A1:M51"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="48.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.140625" style="6" customWidth="1"/>
-    <col min="10" max="10" width="6.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.5703125" style="6" customWidth="1"/>
-    <col min="13" max="13" width="28.42578125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="9.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="6.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" style="5" customWidth="1"/>
+    <col min="13" max="13" width="28.42578125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="M1" s="4" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="A2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="5">
         <v>1</v>
       </c>
-      <c r="E2" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="G2" s="6" t="s">
+      <c r="E2" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C3" s="6" t="s">
+      <c r="A3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="5">
         <v>2</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="A4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>3</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C5" s="6" t="s">
+      <c r="A5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="5">
         <v>4</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="A6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <v>5</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C7" s="6" t="s">
+      <c r="A7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="5">
         <v>6</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="A8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="5">
         <v>7</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C9" s="6" t="s">
+      <c r="A9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="5">
         <v>8</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="6" t="s">
+      <c r="A10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="5">
         <v>9</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" s="6" t="s">
+      <c r="A11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="5">
         <v>10</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" s="6" t="s">
+      <c r="A12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="5">
         <v>11</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="6" t="s">
+      <c r="A13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="5">
         <v>12</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="6" t="s">
+      <c r="A14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="5">
         <v>13</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="6" t="s">
+      <c r="A15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="5">
         <v>14</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="A16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="5">
         <v>15</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C17" s="6" t="s">
+      <c r="A17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="D17" s="6">
+      <c r="D17" s="5">
         <v>16</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C18" s="6" t="s">
+      <c r="A18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D18" s="6">
+      <c r="D18" s="5">
         <v>17</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="6" t="s">
+      <c r="A19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="5">
         <v>18</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C20" s="6" t="s">
+      <c r="A20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D20" s="6">
+      <c r="D20" s="5">
         <v>19</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C21" s="6" t="s">
+      <c r="A21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="5">
         <v>20</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C22" s="6" t="s">
+      <c r="A22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="5">
         <v>21</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C23" s="6" t="s">
+      <c r="A23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="5">
         <v>22</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C24" s="6" t="s">
+      <c r="A24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="5">
         <v>23</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C25" s="6" t="s">
+      <c r="A25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="5">
         <v>24</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E25" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C26" s="6" t="s">
+      <c r="A26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D26" s="6">
+      <c r="D26" s="5">
         <v>25</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C27" s="6" t="s">
+      <c r="A27" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D27" s="6">
+      <c r="D27" s="5">
         <v>1</v>
       </c>
-      <c r="E27" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="G27" s="6" t="s">
+      <c r="E27" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G27" s="5" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C28" s="6" t="s">
+      <c r="A28" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="6">
+      <c r="D28" s="5">
         <v>2</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" s="5" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C29" s="6" t="s">
+      <c r="A29" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D29" s="6">
+      <c r="D29" s="5">
         <v>3</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="5" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C30" s="6" t="s">
+      <c r="A30" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="5">
         <v>4</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C31" s="6" t="s">
+      <c r="A31" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D31" s="6">
+      <c r="D31" s="5">
         <v>5</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C32" s="6" t="s">
+      <c r="A32" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D32" s="6">
+      <c r="D32" s="5">
         <v>6</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C33" s="6" t="s">
+      <c r="A33" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D33" s="6">
+      <c r="D33" s="5">
         <v>7</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C34" s="6" t="s">
+      <c r="A34" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="6">
+      <c r="D34" s="5">
         <v>8</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="E34" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C35" s="6" t="s">
+      <c r="A35" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D35" s="6">
+      <c r="D35" s="5">
         <v>9</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="E35" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C36" s="6" t="s">
+      <c r="A36" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D36" s="6">
+      <c r="D36" s="5">
         <v>10</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="E36" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C37" s="6" t="s">
+      <c r="A37" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D37" s="6">
+      <c r="D37" s="5">
         <v>11</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="E37" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C38" s="6" t="s">
+      <c r="A38" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D38" s="6">
+      <c r="D38" s="5">
         <v>12</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="E38" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C39" s="6" t="s">
+      <c r="A39" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D39" s="6">
+      <c r="D39" s="5">
         <v>13</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="E39" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C40" s="6" t="s">
+      <c r="A40" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D40" s="6">
+      <c r="D40" s="5">
         <v>14</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="E40" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C41" s="6" t="s">
+      <c r="A41" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="D41" s="6">
+      <c r="D41" s="5">
         <v>15</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="E41" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C42" s="6" t="s">
+      <c r="A42" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="D42" s="6">
+      <c r="D42" s="5">
         <v>16</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="E42" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C43" s="6" t="s">
+      <c r="A43" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C43" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D43" s="6">
+      <c r="D43" s="5">
         <v>17</v>
       </c>
-      <c r="E43" s="6" t="s">
+      <c r="E43" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C44" s="6" t="s">
+      <c r="A44" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C44" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D44" s="6">
+      <c r="D44" s="5">
         <v>18</v>
       </c>
-      <c r="E44" s="6" t="s">
+      <c r="E44" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C45" s="6" t="s">
+      <c r="A45" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C45" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D45" s="6">
+      <c r="D45" s="5">
         <v>19</v>
       </c>
-      <c r="E45" s="6" t="s">
+      <c r="E45" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C46" s="6" t="s">
+      <c r="A46" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D46" s="6">
+      <c r="D46" s="5">
         <v>20</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="E46" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B47" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C47" s="6" t="s">
+      <c r="A47" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C47" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D47" s="6">
+      <c r="D47" s="5">
         <v>21</v>
       </c>
-      <c r="E47" s="6" t="s">
+      <c r="E47" s="5" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C48" s="6" t="s">
+      <c r="A48" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D48" s="6">
+      <c r="D48" s="5">
         <v>22</v>
       </c>
-      <c r="E48" s="6" t="s">
+      <c r="E48" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C49" s="6" t="s">
+      <c r="A49" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D49" s="6">
+      <c r="D49" s="5">
         <v>23</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="E49" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C50" s="6" t="s">
+      <c r="A50" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D50" s="6">
+      <c r="D50" s="5">
         <v>24</v>
       </c>
-      <c r="E50" s="6" t="s">
+      <c r="E50" s="5" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C51" s="6" t="s">
+      <c r="A51" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C51" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D51" s="6">
+      <c r="D51" s="5">
         <v>25</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="E51" s="5" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2126,643 +2125,643 @@
   <dimension ref="A1:M144"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="45.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12" style="6" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="45.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="61.140625" style="9" customWidth="1"/>
-    <col min="11" max="11" width="31.85546875" style="6" customWidth="1"/>
-    <col min="12" max="12" width="25.7109375" style="6" customWidth="1"/>
-    <col min="13" max="13" width="32.42578125" style="6" customWidth="1"/>
+    <col min="1" max="1" width="12.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="45.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="61.140625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="31.85546875" style="5" customWidth="1"/>
+    <col min="12" max="12" width="25.7109375" style="5" customWidth="1"/>
+    <col min="13" max="13" width="32.42578125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="K1" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="L1" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="M1" s="6" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="A2" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F2" s="6" t="s">
+      <c r="D2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C3" s="6" t="s">
+      <c r="A3" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F3" s="6" t="s">
+      <c r="D3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C4" s="6" t="s">
+      <c r="A4" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="D4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C5" s="6" t="s">
+      <c r="A5" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="D5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C6" s="6" t="s">
+      <c r="A6" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" s="6" t="s">
+      <c r="D6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C7" s="6" t="s">
+      <c r="A7" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F7" s="6" t="s">
+      <c r="D7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" s="6" t="s">
+      <c r="A8" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F8" s="6" t="s">
+      <c r="D8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C9" s="6" t="s">
+      <c r="A9" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F9" s="6" t="s">
+      <c r="D9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C10" s="6" t="s">
+      <c r="A10" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="6" t="s">
+      <c r="D10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C11" s="6" t="s">
+      <c r="A11" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F11" s="6" t="s">
+      <c r="D11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C12" s="6" t="s">
+      <c r="A12" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F12" s="6" t="s">
+      <c r="D12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C13" s="6" t="s">
+      <c r="A13" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F13" s="6" t="s">
+      <c r="D13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C14" s="6" t="s">
+      <c r="A14" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F14" s="6" t="s">
+      <c r="D14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F14" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G14" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C15" s="6" t="s">
+      <c r="A15" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F15" s="6" t="s">
+      <c r="D15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="G15" s="6" t="s">
+      <c r="G15" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="A16" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F16" s="6" t="s">
+      <c r="D16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="G16" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C17" s="6" t="s">
+      <c r="A17" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F17" s="6" t="s">
+      <c r="D17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C18" s="6" t="s">
+      <c r="A18" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F18" s="6" t="s">
+      <c r="D18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F18" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C19" s="6" t="s">
+      <c r="A19" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F19" s="6" t="s">
+      <c r="D19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="G19" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C20" s="6" t="s">
+      <c r="A20" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F20" s="6" t="s">
+      <c r="D20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F20" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="G20" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C21" s="6" t="s">
+      <c r="A21" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D21" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F21" s="6" t="s">
+      <c r="D21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F21" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="G21" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C22" s="6" t="s">
+      <c r="A22" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F22" s="6" t="s">
+      <c r="D22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G22" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C23" s="6" t="s">
+      <c r="A23" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F23" s="6" t="s">
+      <c r="D23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F23" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="G23" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C24" s="6" t="s">
+      <c r="A24" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D24" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F24" s="6" t="s">
+      <c r="D24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F24" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="G24" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C25" s="6" t="s">
+      <c r="A25" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D25" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" s="6" t="s">
+      <c r="D25" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="G25" s="6" t="s">
+      <c r="G25" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C26" s="6" t="s">
+      <c r="A26" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="D26" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F26" s="6" t="s">
+      <c r="D26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F26" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G26" s="6" t="s">
+      <c r="G26" s="5" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="142" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I142" s="10"/>
-      <c r="J142" s="10"/>
+      <c r="I142" s="9"/>
+      <c r="J142" s="9"/>
     </row>
     <row r="144" spans="9:10" x14ac:dyDescent="0.25">
-      <c r="I144" s="10"/>
-      <c r="J144" s="10"/>
+      <c r="I144" s="9"/>
+      <c r="J144" s="9"/>
     </row>
   </sheetData>
   <dataValidations count="5">

</xml_diff>